<commit_message>
📅 日报更新 2026-08-26 07:04
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-08-26.xlsx
+++ b/data/exports/黄老师/dist_order_2026-08-26.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>49646935</v>
+        <v>49673360</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>49646933</v>
+        <v>49673352</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>49646901</v>
+        <v>49673350</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>49646876</v>
+        <v>49673349</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>49646867</v>
+        <v>49646935</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -425,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>49636232</v>
+        <v>49646933</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -464,7 +464,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
@@ -485,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>49636184</v>
+        <v>49646901</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
@@ -545,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>49636170</v>
+        <v>49646876</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
@@ -605,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>49636157</v>
+        <v>49646867</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
@@ -665,11 +665,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>49593974</v>
+        <v>49636232</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -725,11 +725,11 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>49593671</v>
+        <v>49636184</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -785,11 +785,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>49535916</v>
+        <v>49636170</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
@@ -845,11 +845,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>49535653</v>
+        <v>49636157</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -905,11 +905,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>49535650</v>
+        <v>49593974</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -960,21 +960,16 @@
       <c r="L15" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N15" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>49508265</v>
+        <v>49593671</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>准备1号</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -999,7 +994,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-24 12:49:27</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1030,11 +1025,11 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>49493414</v>
+        <v>49535916</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>真诚</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1059,7 +1054,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-22 23:46:23</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1090,11 +1085,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>49493126</v>
+        <v>49535653</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>如意家电13368134456维修</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1119,7 +1114,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-22 23:28:25</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1150,11 +1145,11 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>49492499</v>
+        <v>49535650</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>莺莺</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1179,7 +1174,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-22 23:27:55</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1205,16 +1200,21 @@
       <c r="L19" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N19" s="0" t="inlineStr">
+        <is>
+          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>49455301</v>
+        <v>49508265</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1270,11 +1270,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>49432023</v>
+        <v>49493414</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1330,11 +1330,11 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>49415939</v>
+        <v>49493126</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>刘盼昭</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-21 22:44:53</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="I22" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
@@ -1390,11 +1390,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>49415918</v>
+        <v>49492499</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>红霞</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-21 22:29:43</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1429,17 +1429,17 @@
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
@@ -1450,11 +1450,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>49415913</v>
+        <v>49455301</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>周开平</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-20 22:46:59</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1489,17 +1489,17 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
@@ -1510,11 +1510,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>49415890</v>
+        <v>49432023</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>花生米</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-20 11:55:45</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1549,37 +1549,32 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K25" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L25" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N25" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>49415874</v>
+        <v>49415939</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>杨梅芳</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1604,7 +1599,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-19 22:48:58</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1635,11 +1630,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>49415871</v>
+        <v>49415918</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>心语无言</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1664,7 +1659,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-19 22:48:24</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1695,59 +1690,304 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
+        <v>49415913</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>安好</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:18</t>
+        </is>
+      </c>
+      <c r="H28" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I28" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J28" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K28" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L28" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" s="0">
+        <v>49415890</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>雨夜聆风</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E29" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F29" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G29" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:56</t>
+        </is>
+      </c>
+      <c r="H29" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I29" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J29" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K29" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L29" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N29" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G30" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H30" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I30" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J30" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K30" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L30" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G31" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H31" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I31" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J31" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K31" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L31" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" s="0">
         <v>49415867</v>
       </c>
-      <c r="B28" s="0" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C28" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D28" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E28" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F28" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G28" s="0" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E32" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G32" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H28" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I28" s="0" t="inlineStr">
+      <c r="H32" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" s="0" t="inlineStr">
         <is>
           <t>黄老师-抖音01</t>
         </is>
       </c>
-      <c r="J28" s="0" t="inlineStr">
+      <c r="J32" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K28" s="0" t="inlineStr">
+      <c r="K32" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L28" s="0" t="inlineStr">
+      <c r="L32" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>